<commit_message>
Added tables in LM,LRU,GCS
</commit_message>
<xml_diff>
--- a/Vajra_Forms_Data_Dictionary.xlsx
+++ b/Vajra_Forms_Data_Dictionary.xlsx
@@ -1252,12 +1252,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
@@ -1593,6 +1593,134 @@
       <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Associated structural sub-system (e.g. Propulsion, Computing, Electrical).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Component/LRU</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>lru_component[]</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (String)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Associated Component/LRU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>lru_qty[]</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (Integer)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Quantity of components.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Part No.</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>lru_part_no[]</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (String)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Part number of the component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Serial no</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>lru_serial_no[]</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (String)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Serial number of the component.</t>
         </is>
       </c>
     </row>
@@ -4250,12 +4378,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
@@ -4305,12 +4433,12 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Serial Number</t>
+          <t>SAP Part number</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>serial_number</t>
+          <t>sap_part_number</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -4320,7 +4448,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Required, Length: 14</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -4330,19 +4458,19 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Unique military grade hardware serial number.</t>
+          <t>14 Digit part no generated on SAP.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Unit Name</t>
+          <t>Customer Part no</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>unit_name</t>
+          <t>customer_part_number</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -4352,7 +4480,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Required, Length: 8</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -4362,171 +4490,363 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Descriptive name for the individual unit (e.g. LM Alpha).</t>
+          <t>08 Digit part no generated for customer.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>Serial Number</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>serial_number</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Unique military grade hardware serial number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Unit Name</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>unit_name</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Descriptive name for the individual unit (e.g. LM Alpha).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>SRLM System</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>srlm_system</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Dropdown (String)</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Read-only (Default: 'LM')</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>LM (Loitering Munition)</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>System categorization, fixed to LM.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>customer_id</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Dropdown (String)</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Acme Rail Systems
 MetroLine Services
 Urban Transit Corp</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Assigns ownership of the unit to a customer.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Contract</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>contract_id</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Dropdown (String)</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>CTR-2024-001
 CTR-2024-014
 CTR-2023-220</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Links the unit deployment to an active contract. Filtered by selected Customer.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Warranty Valid From</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>warranty_valid_from</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Date / String</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Warranty coverage start date (YYYY-MM-DD).</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Warranty Valid To</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>warranty_valid_to</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Date / String</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Warranty coverage end date (YYYY-MM-DD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Component/LRU</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>lm_component[]</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (String)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Associated Component/LRU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Qty aircraft</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>lm_qty[]</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (Integer)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Quantity of components.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Part No.</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>lm_part_no[]</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (String)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Part number of the component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Serial no.</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>lm_serial_no[]</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (String)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Serial number of the component.</t>
         </is>
       </c>
     </row>
@@ -5509,12 +5829,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
@@ -5946,6 +6266,102 @@
       <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Installed software version.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Component/LRU</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>gcs_component[]</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (String)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Associated Component/LRU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Part No.</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>gcs_part_no[]</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (String)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Part number of the component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>gcs_qty[]</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (Integer)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Quantity of components.</t>
         </is>
       </c>
     </row>
@@ -6379,12 +6795,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
@@ -6434,12 +6850,12 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Serial Number</t>
+          <t>SAP Part number</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>serial_number</t>
+          <t>sap_part_number</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -6449,7 +6865,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Required, Length: 14</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -6459,19 +6875,19 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Unique system hardware serial number.</t>
+          <t>14 Digit part no generated on SAP.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Unit Name</t>
+          <t>Customer Part no</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>unit_name</t>
+          <t>customer_part_number</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -6481,7 +6897,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Required, Length: 8</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -6491,171 +6907,427 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Descriptive unit name (e.g. Simulator Prime).</t>
+          <t>08 Digit part no generated for customer.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>Serial Number</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>serial_number</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Unique system hardware serial number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Unit Name</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>unit_name</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Descriptive unit name (e.g. Simulator Prime).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>SRLM System</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>srlm_system</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Dropdown (String)</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Read-only (Default: 'Simulator')</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Simulator</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>System categorization, fixed to Simulator.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>customer_id</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Dropdown (String)</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Acme Rail Systems
 MetroLine Services
 Urban Transit Corp</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Assigns ownership of the simulator to a customer.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Contract</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>contract_id</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Dropdown (String)</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>CTR-2024-001
 CTR-2024-014
 CTR-2023-220</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Links the unit deployment to an active contract. Filtered by selected Customer.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Warranty Valid From</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>warranty_valid_from</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Date / String</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Warranty coverage start date (YYYY-MM-DD).</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Warranty Valid To</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>warranty_valid_to</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Date / String</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Warranty coverage end date (YYYY-MM-DD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Make</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>make</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Manufacturer make.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Manufacturer model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Software version</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>software_version</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Installed software version.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Component/LRU</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>sim_component[]</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (String)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Associated Component/LRU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Part No.</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>sim_part_no[]</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (String)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Part number of the component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>sim_qty[]</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Table Column (Integer)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Required for table row</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Quantity of components.</t>
         </is>
       </c>
     </row>

</xml_diff>